<commit_message>
finish grid credit scoring construction
</commit_message>
<xml_diff>
--- a/outputs/model_selection/best_4_variables_scorecard.xlsx
+++ b/outputs/model_selection/best_4_variables_scorecard.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Score computation" sheetId="1" r:id="R90638f0924054373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model metrics" sheetId="2" r:id="R0ef541ff42334239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Score computation" sheetId="1" r:id="R68d391a4f99b453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model metrics" sheetId="2" r:id="Rd3fcc6bb8c594317"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,8 +14,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="0.00%"/>
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="0.00"/>
+    <x:numFmt numFmtId="201" formatCode="0.00%"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -146,7 +147,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -227,6 +228,12 @@
     <x:xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -247,7 +254,7 @@
     <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -315,12 +322,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -410,6 +463,7 @@
     <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="41.11000061035156" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14.4399995803833" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -430,6 +484,9 @@
       <x:c r="D3" s="9" t="str">
         <x:v>Coeff</x:v>
       </x:c>
+      <x:c r="E3" s="9" t="str">
+        <x:v>Score</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="31.5" customHeight="1">
       <x:c r="A4" s="17" t="n">
@@ -439,10 +496,13 @@
         <x:v>loan_int_rate</x:v>
       </x:c>
       <x:c r="C4" s="21" t="str">
-        <x:v>(12.21, 21.825]</x:v>
+        <x:v>(5.419, 9.91]</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="32" t="n">
+        <x:v>259.05</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="31.5" customHeight="1">
@@ -453,10 +513,13 @@
         <x:v>loan_int_rate</x:v>
       </x:c>
       <x:c r="C5" s="26" t="str">
-        <x:v>(5.419, 9.91]</x:v>
+        <x:v>(9.91, 12.21]</x:v>
       </x:c>
       <x:c r="D5" s="26" t="str">
-        <x:v>1.357044926979 (Coeff_loan_int_rate_1)</x:v>
+        <x:v>0.405083974577 (Coeff_loan_int_rate_2)</x:v>
+      </x:c>
+      <x:c r="E5" s="33" t="n">
+        <x:v>181.72</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="31.5" customHeight="1">
@@ -467,10 +530,13 @@
         <x:v>loan_int_rate</x:v>
       </x:c>
       <x:c r="C6" s="21" t="str">
-        <x:v>(9.91, 12.21]</x:v>
+        <x:v>(12.21, 21.825]</x:v>
       </x:c>
       <x:c r="D6" s="21" t="str">
-        <x:v>0.405083974577 (Coeff_loan_int_rate_2)</x:v>
+        <x:v>1.357044926979 (Coeff_loan_int_rate_1)</x:v>
+      </x:c>
+      <x:c r="E6" s="32" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
@@ -481,10 +547,13 @@
         <x:v>loan_percent_income</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
-        <x:v>(0.2, 0.44]</x:v>
+        <x:v>(-0.001, 0.11]</x:v>
       </x:c>
       <x:c r="D7" s="26" t="str">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="33" t="n">
+        <x:v>307.49</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="31.5" customHeight="1">
@@ -495,10 +564,13 @@
         <x:v>loan_percent_income</x:v>
       </x:c>
       <x:c r="C8" s="21" t="str">
-        <x:v>(-0.001, 0.11]</x:v>
+        <x:v>(0.11, 0.2]</x:v>
       </x:c>
       <x:c r="D8" s="21" t="str">
-        <x:v>1.610830556754 (Coeff_loan_percent_income_1)</x:v>
+        <x:v>0.190140541733 (Coeff_loan_percent_income_2)</x:v>
+      </x:c>
+      <x:c r="E8" s="32" t="n">
+        <x:v>271.2</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="31.5" customHeight="1">
@@ -509,10 +581,13 @@
         <x:v>loan_percent_income</x:v>
       </x:c>
       <x:c r="C9" s="26" t="str">
-        <x:v>(0.11, 0.2]</x:v>
+        <x:v>(0.2, 0.44]</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
-        <x:v>0.190140541733 (Coeff_loan_percent_income_2)</x:v>
+        <x:v>1.610830556754 (Coeff_loan_percent_income_1)</x:v>
+      </x:c>
+      <x:c r="E9" s="33" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="31.5" customHeight="1">
@@ -528,6 +603,9 @@
       <x:c r="D10" s="21" t="str">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="E10" s="32" t="n">
+        <x:v>59.52</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="31.5" customHeight="1">
       <x:c r="A11" s="17" t="n">
@@ -542,6 +620,9 @@
       <x:c r="D11" s="26" t="str">
         <x:v>0.311775358054 (Coeff_cb_person_default_on_file_Y)</x:v>
       </x:c>
+      <x:c r="E11" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="31.5" customHeight="1">
       <x:c r="A12" s="17" t="n">
@@ -556,6 +637,9 @@
       <x:c r="D12" s="21" t="str">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="E12" s="32" t="n">
+        <x:v>373.94</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="31.5" customHeight="1">
       <x:c r="A13" s="17" t="n">
@@ -570,6 +654,9 @@
       <x:c r="D13" s="26" t="str">
         <x:v>0.959293765716 (Coeff_home_ownership_3_MORTGAGE)</x:v>
       </x:c>
+      <x:c r="E13" s="33" t="n">
+        <x:v>190.82</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="31.5" customHeight="1">
       <x:c r="A14" s="17" t="n">
@@ -584,6 +671,9 @@
       <x:c r="D14" s="21" t="str">
         <x:v>1.958944283424 (Coeff_home_ownership_3_OTHER_RENT)</x:v>
       </x:c>
+      <x:c r="E14" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="25.5" customHeight="1">
       <x:c r="A15" s="29" t="str">
@@ -598,10 +688,11 @@
       <x:c r="D15" s="26" t="n">
         <x:v>-4.243875750401388</x:v>
       </x:c>
+      <x:c r="E15" s="33" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A1:E1"/>
     <x:mergeCell ref="A15:C15"/>
     <x:mergeCell ref="A4:A6"/>
     <x:mergeCell ref="B4:B6"/>
@@ -625,95 +716,95 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="32" t="str">
+      <x:c r="A1" s="34" t="str">
         <x:v>Selected 4-variable model</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="35" t="str">
+      <x:c r="A3" s="37" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="B3" s="35" t="str">
+      <x:c r="B3" s="37" t="str">
         <x:v>Value</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="41" t="str">
+      <x:c r="A4" s="43" t="str">
         <x:v>Formula</x:v>
       </x:c>
-      <x:c r="B4" s="39" t="str">
+      <x:c r="B4" s="41" t="str">
         <x:v>Q("def") ~ C(Q("loan_int_rate_dis"), Treatment(reference=3)) + C(Q("loan_percent_income_dis"), Treatment(reference=3)) + C(Q("cb_person_default_on_file"), Treatment(reference='N')) + C(Q("home_ownership_3"), Treatment(reference='OWN'))</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="41" t="str">
+      <x:c r="A5" s="43" t="str">
         <x:v>Target</x:v>
       </x:c>
-      <x:c r="B5" s="39" t="str">
+      <x:c r="B5" s="41" t="str">
         <x:v>def</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="41" t="str">
+      <x:c r="A6" s="43" t="str">
         <x:v>Variables</x:v>
       </x:c>
-      <x:c r="B6" s="39" t="str">
+      <x:c r="B6" s="41" t="str">
         <x:v>loan_int_rate_dis, loan_percent_income_dis, cb_person_default_on_file, home_ownership_3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="41" t="str">
+      <x:c r="A7" s="43" t="str">
         <x:v>Gini train</x:v>
       </x:c>
-      <x:c r="B7" s="42" t="n">
+      <x:c r="B7" s="44" t="n">
         <x:v>0.5938156050410457</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="41" t="str">
+      <x:c r="A8" s="43" t="str">
         <x:v>Gini test</x:v>
       </x:c>
-      <x:c r="B8" s="42" t="n">
+      <x:c r="B8" s="44" t="n">
         <x:v>0.5804011103284024</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="41" t="str">
+      <x:c r="A9" s="43" t="str">
         <x:v>Gini OOT</x:v>
       </x:c>
-      <x:c r="B9" s="42" t="n">
+      <x:c r="B9" s="44" t="n">
         <x:v>0.5740931994207759</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="41" t="str">
+      <x:c r="A10" s="43" t="str">
         <x:v>Gini penalized</x:v>
       </x:c>
-      <x:c r="B10" s="42" t="n">
+      <x:c r="B10" s="44" t="n">
         <x:v>0.5600679100133259</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="41" t="str">
+      <x:c r="A11" s="43" t="str">
         <x:v>Recall penalized</x:v>
       </x:c>
-      <x:c r="B11" s="42" t="n">
+      <x:c r="B11" s="44" t="n">
         <x:v>0.2261151956813736</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="41" t="str">
+      <x:c r="A12" s="43" t="str">
         <x:v>F1 penalized</x:v>
       </x:c>
-      <x:c r="B12" s="42" t="n">
+      <x:c r="B12" s="44" t="n">
         <x:v>0.3350962546214514</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="41" t="str">
+      <x:c r="A13" s="43" t="str">
         <x:v>PR AUC penalized</x:v>
       </x:c>
-      <x:c r="B13" s="42" t="n">
+      <x:c r="B13" s="44" t="n">
         <x:v>0.4843832102478143</x:v>
       </x:c>
     </x:row>

</xml_diff>